<commit_message>
updated campaigns so the brightness logit > 0.5
</commit_message>
<xml_diff>
--- a/design-campaign-EGFP/shortlists/shortlist_EBFP_DMS-guide.xlsx
+++ b/design-campaign-EGFP/shortlists/shortlist_EBFP_DMS-guide.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="shortlist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'shortlist'!$A$1:$O$13</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -425,8 +427,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="43" customWidth="1" min="13" max="13"/>
+    <col width="44" customWidth="1" min="14" max="14"/>
+    <col width="44" customWidth="1" min="15" max="15"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -471,25 +490,35 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>n_mut_vs_EGFP</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>is_id</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>is_bright</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>bright_logit</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>aa_sequence</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>dna_sequence</t>
         </is>
@@ -516,15 +545,19 @@
       </c>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKFICTTGKLPVPWPTLVTTLTYGVQCFSRYPDHMKQHDFFKSAMPEGYVQERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNYNSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAATTTATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGACCACCCTGACCTATGGCGTGCAGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCTATGTGCAGGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACTATAACAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
@@ -551,15 +584,19 @@
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
         <is>
           <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKFICTTGKLPVPWPTLVTTLTHGVQCFSRYPDHMKQHDFFKSAMPEGYVQERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNFNSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAATTTATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGACCACCCTGACCCATGGCGTGCAGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCTATGTGCAGGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACTTTAACAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
@@ -594,25 +631,33 @@
       <c r="H4" t="n">
         <v>451.1</v>
       </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+      <c r="I4" t="n">
+        <v>9</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
         <v>2.21</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>designs_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
         <is>
           <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTIKVICTTGKLPVPWPTLVSTLSYGVACFSRYPDHMKQHDFFKSAMPEGVVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGISHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCATTAAAGTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCGTGGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCATTAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
@@ -647,25 +692,33 @@
       <c r="H5" t="n">
         <v>458.9</v>
       </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+      <c r="I5" t="n">
+        <v>10</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
         <v>2.81</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>designs_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
         <is>
           <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTIKAICTTGKLPVPWPTLVSTLSYGVACFSRYPDHMKQHDFFKSAMPEGSVYERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGVSHNIYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCATTAAAGCGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCAGCGTGTATGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCGTGAGCCATAACATTTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
@@ -695,32 +748,40 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="n">
-        <v>406</v>
+        <v>395.3</v>
       </c>
       <c r="H6" t="n">
-        <v>465.5</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>467</v>
+      </c>
+      <c r="I6" t="n">
+        <v>11</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K6" t="n">
-        <v>2.69</v>
-      </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGIVSERTIFFKDDGNYKTRAEVKFEGDTLVSRIELKGIDFKEDGNILGHKLEYNDSSHNYYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0.78</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCATTGTGAGCGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAGCCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGATAGCAGCCATAACTATTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>lam-ex20_lam-em20_lam-bright40_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGTTCFSRYPDHMKQHDFFKSAMPEGLVKERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGKSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCACCACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGAAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCAAAAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -748,32 +809,40 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="n">
-        <v>406.3</v>
+        <v>400.2</v>
       </c>
       <c r="H7" t="n">
-        <v>466.7</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>462.3</v>
+      </c>
+      <c r="I7" t="n">
+        <v>11</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K7" t="n">
-        <v>2.63</v>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKITIKAICTTGKLPVPWPTLVSTLSYGVACFSRYPDHMKQHDFFKSAMPEGEVQERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGLSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0.72</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAAATTACCATTAAAGCGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCGAAGTGCAGGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCCTGAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>lam-ex20_lam-em20_lam-bright40_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTVKIICTTGKLPVPWPTLVATFSYGVACFSRYPDHMKQHDFFKSAMPEGLVEERTIFFKDDGNYKTRAEVKFEGDTLVTRIELKGIDFKEDGNILGHKLEYNGESHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCGTGAAAATTATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGGCGACCTTTAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGACCCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCGAAAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -801,32 +870,40 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="n">
-        <v>403.3</v>
+        <v>401</v>
       </c>
       <c r="H8" t="n">
-        <v>470.1</v>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>464.7</v>
+      </c>
+      <c r="I8" t="n">
+        <v>9</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGFVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNTGSHNYYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>2.51</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCTTTGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACACCGGCAGCCATAACTATTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>lam-ex20_lam-em20_lam-bright40_lam-edit15</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKVTLKVICTTGKLPVPWPTLVSTLSYGVSCFSRYPDHMKQHDFFKSAMPEGLVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGESHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAAGTGACCCTGAAAGTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGAGCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCGAAAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -854,32 +931,40 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
-        <v>406.5</v>
+        <v>405.9</v>
       </c>
       <c r="H9" t="n">
-        <v>468.4</v>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>464.2</v>
+      </c>
+      <c r="I9" t="n">
+        <v>12</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K9" t="n">
-        <v>5.33</v>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLVSTLSYGVACFSRYPDHMKQHDFFKSAMPEGVVTERTIFFKDDGNYKTRAEVKFEGDTLVSRIELKGIDFKEDGNILGHKLEYNERSHNIYIMADKQKNGIKVNAKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>1.02</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCGTGGTGACCGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAGCCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGAACGCAGCCATAACATTTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACGCGAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>lam-ex30_lam-em30_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLVSSLSYGTVCFSRYPDHMKQHDFFKSAMPEGIVEERTIFFKDDGNYKTRAEVKFEGDTLVSRIELKGIDFKEDGNILGHKLEYNDESHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCAGCCTGAGCTATGGCACCGTGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCATTGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAGCCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGATGAAAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -907,32 +992,40 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="n">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="H10" t="n">
-        <v>464.4</v>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>465.5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>12</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K10" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLVSSLSYGVACFSRYPDHMKQHDFFKSAMPEGIVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNKNSTNYYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>2.69</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCAGCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCATTGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACAAAAACAGCACCAACTATTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>designs_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGIVSERTIFFKDDGNYKTRAEVKFEGDTLVSRIELKGIDFKEDGNILGHKLEYNDSSHNYYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCATTGTGAGCGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAGCCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGATAGCAGCCATAACTATTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -960,32 +1053,40 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
-        <v>405</v>
+        <v>405.9</v>
       </c>
       <c r="H11" t="n">
-        <v>471.2</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>466.3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K11" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="L11" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVACFSRYPDHMKQHDFFKSAMPEGLVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNKSSHNVYIMADKQKNGIKVNAKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>1.88</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACAAAAGCAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACGCGAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>lam-ex20_lam-em20_lam-bright40_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGLVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNDNSTNFYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGATAACAGCACCAACTTTTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -1013,32 +1114,40 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
-        <v>412</v>
+        <v>406.3</v>
       </c>
       <c r="H12" t="n">
-        <v>464.4</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>466.7</v>
+      </c>
+      <c r="I12" t="n">
+        <v>9</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K12" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTIKAICTTGKLPVPWPTLVATLSYGVACFSRYPDHMKQHDFFKSAMPEGLVHERTIFFKDDGNYKTRAEVKFEGDTLVARIELKGIDFKEDGNILGHKLEYNKLSHNIYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>2.63</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCATTAAAGCGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGGCGACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCCTGGTGCATGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGGCGCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACAAACTGAGCCATAACATTTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>designs_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKITIKAICTTGKLPVPWPTLVSTLSYGVACFSRYPDHMKQHDFFKSAMPEGEVQERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNGLSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQSALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAAATTACCATTAAAGCGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGGTGAGCACCCTGAGCTATGGCGTGGCGTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCGAAGTGCAGGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGGCCTGAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGAGCGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
@@ -1066,36 +1175,45 @@
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>411</v>
+        <v>403.3</v>
       </c>
       <c r="H13" t="n">
-        <v>465.4</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
+        <v>470.1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>11</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="K13" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="L13" t="inlineStr">
-        <is>
-          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTVKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGVVTERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNDKSHNVYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
-        </is>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>1.2</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCGTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCGTGGTGACCGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACGATAAAAGCCATAACGTGTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
+          <t>designs_lam-bright60_lam-edit10</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>MVSKGEELFTGVVPILVELDGDVNGHKFSVSGEGEGDATYGKLTLKLICTTGKLPVPWPTLLSTLSYGVTCFSRYPDHMKQHDFFKSAMPEGFVEERTIFFKDDGNYKTRAEVKFEGDTLVNRIELKGIDFKEDGNILGHKLEYNTGSHNYYIMADKQKNGIKVNFKIRHNIEDGSVQLADHYQQNTPIGDGPVLLPDNHYLSTQAALSKDPNEKRDHMVLLEFVTAAGITLGMDELYK</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>ATGGTGAGCAAAGGCGAAGAACTGTTTACCGGCGTGGTGCCGATTCTGGTGGAACTGGATGGCGATGTGAACGGCCATAAATTTAGCGTGAGCGGCGAAGGCGAAGGCGATGCGACCTATGGCAAACTGACCCTGAAACTGATTTGCACCACCGGCAAACTGCCGGTGCCGTGGCCGACCCTGCTGAGCACCCTGAGCTATGGCGTGACCTGCTTTAGCCGCTATCCGGATCATATGAAACAGCATGATTTTTTTAAAAGCGCGATGCCGGAAGGCTTTGTGGAAGAACGCACCATTTTTTTTAAAGATGATGGCAACTATAAAACCCGCGCGGAAGTGAAATTTGAAGGCGATACCCTGGTGAACCGCATTGAACTGAAAGGCATTGATTTTAAAGAAGATGGCAACATTCTGGGCCATAAACTGGAATATAACACCGGCAGCCATAACTATTATATTATGGCGGATAAACAGAAAAACGGCATTAAAGTGAACTTTAAAATTCGCCATAACATTGAAGATGGCAGCGTGCAGCTGGCGGATCATTATCAGCAGAACACCCCGATTGGCGATGGCCCGGTGCTGCTGCCGGATAACCATTATCTGAGCACCCAGGCGGCGCTGAGCAAAGATCCGAACGAAAAACGCGATCATATGGTGCTGCTGGAATTTGTGACCGCGGCGGGCATTACCCTGGGCATGGATGAACTGTATAAATAA</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>